<commit_message>
feat: add merged phase column to PAB schedule
Insert 阶段 as column A and merge first-phase vs second-phase rows
so the sheet groups PAB060–142 and PAB180–220 at a glance.

Co-authored-by: zer2803-cloud <zer2803-cloud@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PAB产品计划表.xlsx
+++ b/PAB产品计划表.xlsx
@@ -10,7 +10,7 @@
     <sheet name="时间节点计划表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'时间节点计划表'!$A$1:$F$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'时间节点计划表'!$A$1:$G$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,11 +42,17 @@
     </font>
     <font>
       <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
       <color rgb="006B7280"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,8 +69,18 @@
         <fgColor rgb="00F3F7FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEBD0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -86,13 +102,49 @@
         <color rgb="00B7C9D6"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9D6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C9D6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C9D6"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B7C9D6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -113,7 +165,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,44 +551,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>阶段</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>任务摘要</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>预估完成节点</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>实际完成节点</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>超时原因</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>任务责任人</t>
         </is>
@@ -542,994 +603,1048 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>第一期</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
           <t>第一期·零件图纸整理归档</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>四批型号单级和双级所涉零件图纸整理完毕并分类归档。范围：PAB060、PAB090、PAB115、PAB142。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="D2" s="4" t="n">
         <v>46258</v>
       </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>第一期·零件下单采购</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>各零件形成采购表单并填写数量，单级和双级各10台。范围：PAB060、PAB090、PAB115、PAB142。</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="D3" s="7" t="n">
         <v>46259</v>
       </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>第一期·标准件下单采购</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>各标准件形成采购表单并填写数量。范围：PAB060、PAB090、PAB115、PAB142。</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>46259</v>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>装配线布局</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>装配线布局完成。协助人：吴金平、王杰、吴晨阳。</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="D5" s="7" t="n">
         <v>46280</v>
       </c>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>莫华华</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>装配工具到位</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>轴用卡钳、孔用卡钳、镊子、压机、润滑脂、螺纹禁锢胶、密封厌氧胶等装配工具到位。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="D6" s="4" t="n">
         <v>46275</v>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>吴晨阳</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>PAB060·零件到位</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>PAB060 零件到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="D7" s="7" t="n">
         <v>46289</v>
       </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>PAB060·工装图纸绘制</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>PAB060 工装图纸绘制完成。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>46262</v>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>PAB060·工装实物到位</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>PAB060 工装实物到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="D9" s="7" t="n">
         <v>46280</v>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>PAB060·排针机安装调试</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>排针机1安装到位并调试完毕。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="D10" s="4" t="n">
         <v>46289</v>
       </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>吴金平</t>
         </is>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>PAB060·单级样机</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>完成 PAB060 单级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="D11" s="7" t="n">
         <v>46291</v>
       </c>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>PAB060·双级样机</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>完成 PAB060 双级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="D12" s="4" t="n">
         <v>46293</v>
       </c>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>PAB090·零件到位</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>PAB090 零件到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="D13" s="7" t="n">
         <v>46292</v>
       </c>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>PAB090·工装图纸绘制</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>PAB090 工装图纸绘制完成。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="D14" s="4" t="n">
         <v>46266</v>
       </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>PAB090·工装实物到位</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>PAB090 工装实物到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="D15" s="7" t="n">
         <v>46285</v>
       </c>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>PAB090·排针机安装调试</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>排针机1安装到位并调试完毕。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="D16" s="4" t="n">
         <v>46292</v>
       </c>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>吴金平</t>
         </is>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>PAB090·单级样机</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>完成 PAB090 单级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="D17" s="7" t="n">
         <v>46294</v>
       </c>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="5" t="inlineStr"/>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>PAB090·双级样机</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>完成 PAB090 双级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="D18" s="4" t="n">
         <v>46295</v>
       </c>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>PAB115·零件到位</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>PAB115 零件到位（原文标注：国庆假期）。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="D19" s="7" t="n">
         <v>46303</v>
       </c>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>PAB115·工装图纸绘制</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>PAB115 工装图纸绘制完成。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="D20" s="4" t="n">
         <v>46269</v>
       </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>PAB115·工装实物到位</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>PAB115 工装实物到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="D21" s="7" t="n">
         <v>46290</v>
       </c>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="5" t="inlineStr"/>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>PAB115·排针机安装调试</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>排针机1安装到位并调试完毕。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="D22" s="4" t="n">
         <v>46303</v>
       </c>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>吴金平</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>PAB115·单级样机</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>完成 PAB115 单级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="D23" s="7" t="n">
         <v>46304</v>
       </c>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>PAB115·双级样机</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>完成 PAB115 双级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="D24" s="4" t="n">
         <v>46306</v>
       </c>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>PAB142·零件到位</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>PAB142 零件到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="D25" s="7" t="n">
         <v>46307</v>
       </c>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="5" t="inlineStr"/>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>PAB142·工装图纸绘制</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>PAB142 工装图纸绘制完成。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="D26" s="4" t="n">
         <v>46269</v>
       </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>PAB142·工装实物到位</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>PAB142 工装实物到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="D27" s="7" t="n">
         <v>46294</v>
       </c>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="5" t="inlineStr"/>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>PAB142·排针机安装调试</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>排针机1、排针机2安装到位并调试完毕。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="D28" s="4" t="n">
         <v>46307</v>
       </c>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>吴金平</t>
         </is>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>PAB142·单级样机</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>完成 PAB142 单级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="D29" s="7" t="n">
         <v>46308</v>
       </c>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="5" t="inlineStr"/>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="6" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>PAB142·双级样机</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>完成 PAB142 双级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="D30" s="4" t="n">
         <v>46310</v>
       </c>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>第二期</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>第二期·零件图纸整理归档</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>四批型号单级和双级所涉零件图纸整理完毕并分类归档。范围：PAB180、PAB220。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="D31" s="7" t="n">
         <v>46272</v>
       </c>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="5" t="inlineStr"/>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="9" t="n"/>
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>第二期·零件下单采购</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>各零件形成采购表单并填写数量，单级和双级各10台。范围：PAB180、PAB220。</t>
         </is>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="D32" s="4" t="n">
         <v>46275</v>
       </c>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>第二期·标准件下单采购</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>各标准件形成采购表单并填写数量。范围：PAB180、PAB220。</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="D33" s="7" t="n">
         <v>46275</v>
       </c>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="5" t="inlineStr"/>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="6" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="9" t="n"/>
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>PAB180·零件到位</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>PAB180 零件到位（原文标注：国庆假期）。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="D34" s="4" t="n">
         <v>46310</v>
       </c>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="9" t="n"/>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>PAB180·工装图纸绘制</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>PAB180 工装图纸绘制完成。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="D35" s="7" t="n">
         <v>46276</v>
       </c>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="5" t="inlineStr"/>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="6" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="9" t="n"/>
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>PAB180·工装实物到位</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>PAB180 工装实物到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="D36" s="4" t="n">
         <v>46303</v>
       </c>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>PAB180·排针机安装调试</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>排针机1、排针机2安装到位并调试完毕。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="D37" s="7" t="n">
         <v>46310</v>
       </c>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="6" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr">
         <is>
           <t>吴金平</t>
         </is>
       </c>
     </row>
     <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="9" t="n"/>
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>PAB180·单级样机</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>完成 PAB180 单级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="D38" s="4" t="n">
         <v>46311</v>
       </c>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>PAB180·双级样机</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>完成 PAB180 双级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C39" s="6" t="n">
+      <c r="D39" s="7" t="n">
         <v>46314</v>
       </c>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>PAB220·零件到位</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>PAB220 零件到位（原文标注：国庆假期）。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="D40" s="4" t="n">
         <v>46315</v>
       </c>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="3" t="inlineStr"/>
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="9" t="n"/>
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>PAB220·工装图纸绘制</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>PAB220 工装图纸绘制完成。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C41" s="6" t="n">
+      <c r="D41" s="7" t="n">
         <v>46279</v>
       </c>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="5" t="inlineStr"/>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="9" t="n"/>
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>PAB220·工装实物到位</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>PAB220 工装实物到位。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="D42" s="4" t="n">
         <v>46305</v>
       </c>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="3" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="9" t="n"/>
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>PAB220·排针机安装调试</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>排针机1、排针机2安装到位并调试完毕。协助人：王杰。</t>
         </is>
       </c>
-      <c r="C43" s="6" t="n">
+      <c r="D43" s="7" t="n">
         <v>46315</v>
       </c>
-      <c r="D43" s="7" t="n"/>
-      <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="6" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
         <is>
           <t>吴金平</t>
         </is>
       </c>
     </row>
     <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="9" t="n"/>
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>PAB220·单级样机</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>完成 PAB220 单级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="D44" s="4" t="n">
         <v>46316</v>
       </c>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="3" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="9" t="n"/>
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>PAB220·双级样机</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>完成 PAB220 双级样机。协助人：吴晨阳。</t>
         </is>
       </c>
-      <c r="C45" s="6" t="n">
+      <c r="D45" s="7" t="n">
         <v>46318</v>
       </c>
-      <c r="D45" s="7" t="n"/>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr">
         <is>
           <t>王杰</t>
         </is>
       </c>
     </row>
     <row r="47" ht="40" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>说明：数据来自《PAB产品计划表》Word原文。原文仅有预估节点，实际完成节点留空待填；填写后若实际完成节点晚于预估完成节点，D列单元格自动红色底纹。协助人写入任务摘要；任务责任人取原文「责任人」。</t>
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>说明：数据来自《PAB产品计划表》Word原文。A列按第一期/第二期合并。原文仅有预估节点，实际完成节点留空待填；填写后若实际完成节点晚于预估完成节点，E列单元格自动红色底纹。协助人写入任务摘要；任务责任人取原文「责任人」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F45">
-    <sortState ref="A1:F45">
-      <sortCondition descending="0" ref="C2:C45"/>
+  <autoFilter ref="A1:G45">
+    <sortState ref="A1:G45">
+      <sortCondition descending="0" ref="D2:D45"/>
     </sortState>
   </autoFilter>
-  <mergeCells count="1">
-    <mergeCell ref="A47:F47"/>
+  <mergeCells count="3">
+    <mergeCell ref="A31:A45"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A2:A30"/>
   </mergeCells>
-  <conditionalFormatting sqref="D2:D200">
+  <conditionalFormatting sqref="E2:E200">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(ISNUMBER(D2),ISNUMBER(C2),D2&gt;C2)</formula>
+      <formula>AND(ISNUMBER(E2),ISNUMBER(D2),E2&gt;D2)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="D2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: restore Gantt planned dates hidden by empty-string IF
WPS/Excel can treat a date as equal to \"\", so IF(E=\"\", \"\", E)
wrote blanks into column D. Bars then failed ISNUMBER($D). Quote
planned dates directly from the main sheet and drop extra CF on D.

Co-authored-by: zer2803-cloud <zer2803-cloud@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PAB产品计划表.xlsx
+++ b/PAB产品计划表.xlsx
@@ -325,7 +325,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="7">
     <dxf>
       <font>
         <name val="微软雅黑"/>
@@ -413,59 +413,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFA9D08E"/>
           <bgColor rgb="FFA9D08E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <color rgb="001F2937"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6EAF8"/>
-          <bgColor rgb="FFD6EAF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <b val="1"/>
-        <color rgb="00991B1B"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFECACA"/>
-          <bgColor rgb="FFFECACA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <color rgb="0014532D"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBBF7D0"/>
-          <bgColor rgb="FFBBF7D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <color rgb="001F2937"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFDE68A"/>
-          <bgColor rgb="FFFDE68A"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3222,11 +3169,11 @@
         </is>
       </c>
       <c r="D3" s="23">
-        <f>IF('时间节点计划表'!E2="","",'时间节点计划表'!E2)</f>
+        <f>'时间节点计划表'!E2</f>
         <v/>
       </c>
       <c r="E3" s="23">
-        <f>IF('时间节点计划表'!F2="","",'时间节点计划表'!F2)</f>
+        <f>IF(COUNT('时间节点计划表'!F2),'时间节点计划表'!F2,"")</f>
         <v/>
       </c>
       <c r="F3" s="24" t="inlineStr"/>
@@ -3492,11 +3439,11 @@
         </is>
       </c>
       <c r="D4" s="28">
-        <f>IF('时间节点计划表'!E2="","",'时间节点计划表'!E2)</f>
+        <f>'时间节点计划表'!E2</f>
         <v/>
       </c>
       <c r="E4" s="28">
-        <f>IF('时间节点计划表'!F2="","",'时间节点计划表'!F2)</f>
+        <f>IF(COUNT('时间节点计划表'!F2),'时间节点计划表'!F2,"")</f>
         <v/>
       </c>
       <c r="F4" s="29">
@@ -3765,11 +3712,11 @@
         </is>
       </c>
       <c r="D5" s="23">
-        <f>IF('时间节点计划表'!E3="","",'时间节点计划表'!E3)</f>
+        <f>'时间节点计划表'!E3</f>
         <v/>
       </c>
       <c r="E5" s="23">
-        <f>IF('时间节点计划表'!F3="","",'时间节点计划表'!F3)</f>
+        <f>IF(COUNT('时间节点计划表'!F3),'时间节点计划表'!F3,"")</f>
         <v/>
       </c>
       <c r="F5" s="24" t="inlineStr"/>
@@ -4035,11 +3982,11 @@
         </is>
       </c>
       <c r="D6" s="28">
-        <f>IF('时间节点计划表'!E3="","",'时间节点计划表'!E3)</f>
+        <f>'时间节点计划表'!E3</f>
         <v/>
       </c>
       <c r="E6" s="28">
-        <f>IF('时间节点计划表'!F3="","",'时间节点计划表'!F3)</f>
+        <f>IF(COUNT('时间节点计划表'!F3),'时间节点计划表'!F3,"")</f>
         <v/>
       </c>
       <c r="F6" s="29">
@@ -4308,11 +4255,11 @@
         </is>
       </c>
       <c r="D7" s="23">
-        <f>IF('时间节点计划表'!E4="","",'时间节点计划表'!E4)</f>
+        <f>'时间节点计划表'!E4</f>
         <v/>
       </c>
       <c r="E7" s="23">
-        <f>IF('时间节点计划表'!F4="","",'时间节点计划表'!F4)</f>
+        <f>IF(COUNT('时间节点计划表'!F4),'时间节点计划表'!F4,"")</f>
         <v/>
       </c>
       <c r="F7" s="24" t="inlineStr"/>
@@ -4578,11 +4525,11 @@
         </is>
       </c>
       <c r="D8" s="28">
-        <f>IF('时间节点计划表'!E4="","",'时间节点计划表'!E4)</f>
+        <f>'时间节点计划表'!E4</f>
         <v/>
       </c>
       <c r="E8" s="28">
-        <f>IF('时间节点计划表'!F4="","",'时间节点计划表'!F4)</f>
+        <f>IF(COUNT('时间节点计划表'!F4),'时间节点计划表'!F4,"")</f>
         <v/>
       </c>
       <c r="F8" s="29">
@@ -4851,11 +4798,11 @@
         </is>
       </c>
       <c r="D9" s="23">
-        <f>IF('时间节点计划表'!E5="","",'时间节点计划表'!E5)</f>
+        <f>'时间节点计划表'!E5</f>
         <v/>
       </c>
       <c r="E9" s="23">
-        <f>IF('时间节点计划表'!F5="","",'时间节点计划表'!F5)</f>
+        <f>IF(COUNT('时间节点计划表'!F5),'时间节点计划表'!F5,"")</f>
         <v/>
       </c>
       <c r="F9" s="24" t="inlineStr"/>
@@ -5121,11 +5068,11 @@
         </is>
       </c>
       <c r="D10" s="28">
-        <f>IF('时间节点计划表'!E5="","",'时间节点计划表'!E5)</f>
+        <f>'时间节点计划表'!E5</f>
         <v/>
       </c>
       <c r="E10" s="28">
-        <f>IF('时间节点计划表'!F5="","",'时间节点计划表'!F5)</f>
+        <f>IF(COUNT('时间节点计划表'!F5),'时间节点计划表'!F5,"")</f>
         <v/>
       </c>
       <c r="F10" s="29">
@@ -5394,11 +5341,11 @@
         </is>
       </c>
       <c r="D11" s="23">
-        <f>IF('时间节点计划表'!E6="","",'时间节点计划表'!E6)</f>
+        <f>'时间节点计划表'!E6</f>
         <v/>
       </c>
       <c r="E11" s="23">
-        <f>IF('时间节点计划表'!F6="","",'时间节点计划表'!F6)</f>
+        <f>IF(COUNT('时间节点计划表'!F6),'时间节点计划表'!F6,"")</f>
         <v/>
       </c>
       <c r="F11" s="24" t="inlineStr"/>
@@ -5664,11 +5611,11 @@
         </is>
       </c>
       <c r="D12" s="28">
-        <f>IF('时间节点计划表'!E6="","",'时间节点计划表'!E6)</f>
+        <f>'时间节点计划表'!E6</f>
         <v/>
       </c>
       <c r="E12" s="28">
-        <f>IF('时间节点计划表'!F6="","",'时间节点计划表'!F6)</f>
+        <f>IF(COUNT('时间节点计划表'!F6),'时间节点计划表'!F6,"")</f>
         <v/>
       </c>
       <c r="F12" s="29">
@@ -5937,11 +5884,11 @@
         </is>
       </c>
       <c r="D13" s="23">
-        <f>IF('时间节点计划表'!E7="","",'时间节点计划表'!E7)</f>
+        <f>'时间节点计划表'!E7</f>
         <v/>
       </c>
       <c r="E13" s="23">
-        <f>IF('时间节点计划表'!F7="","",'时间节点计划表'!F7)</f>
+        <f>IF(COUNT('时间节点计划表'!F7),'时间节点计划表'!F7,"")</f>
         <v/>
       </c>
       <c r="F13" s="24" t="inlineStr"/>
@@ -6207,11 +6154,11 @@
         </is>
       </c>
       <c r="D14" s="28">
-        <f>IF('时间节点计划表'!E7="","",'时间节点计划表'!E7)</f>
+        <f>'时间节点计划表'!E7</f>
         <v/>
       </c>
       <c r="E14" s="28">
-        <f>IF('时间节点计划表'!F7="","",'时间节点计划表'!F7)</f>
+        <f>IF(COUNT('时间节点计划表'!F7),'时间节点计划表'!F7,"")</f>
         <v/>
       </c>
       <c r="F14" s="29">
@@ -6480,11 +6427,11 @@
         </is>
       </c>
       <c r="D15" s="23">
-        <f>IF('时间节点计划表'!E8="","",'时间节点计划表'!E8)</f>
+        <f>'时间节点计划表'!E8</f>
         <v/>
       </c>
       <c r="E15" s="23">
-        <f>IF('时间节点计划表'!F8="","",'时间节点计划表'!F8)</f>
+        <f>IF(COUNT('时间节点计划表'!F8),'时间节点计划表'!F8,"")</f>
         <v/>
       </c>
       <c r="F15" s="24" t="inlineStr"/>
@@ -6750,11 +6697,11 @@
         </is>
       </c>
       <c r="D16" s="28">
-        <f>IF('时间节点计划表'!E8="","",'时间节点计划表'!E8)</f>
+        <f>'时间节点计划表'!E8</f>
         <v/>
       </c>
       <c r="E16" s="28">
-        <f>IF('时间节点计划表'!F8="","",'时间节点计划表'!F8)</f>
+        <f>IF(COUNT('时间节点计划表'!F8),'时间节点计划表'!F8,"")</f>
         <v/>
       </c>
       <c r="F16" s="29">
@@ -7023,11 +6970,11 @@
         </is>
       </c>
       <c r="D17" s="23">
-        <f>IF('时间节点计划表'!E9="","",'时间节点计划表'!E9)</f>
+        <f>'时间节点计划表'!E9</f>
         <v/>
       </c>
       <c r="E17" s="23">
-        <f>IF('时间节点计划表'!F9="","",'时间节点计划表'!F9)</f>
+        <f>IF(COUNT('时间节点计划表'!F9),'时间节点计划表'!F9,"")</f>
         <v/>
       </c>
       <c r="F17" s="24" t="inlineStr"/>
@@ -7293,11 +7240,11 @@
         </is>
       </c>
       <c r="D18" s="28">
-        <f>IF('时间节点计划表'!E9="","",'时间节点计划表'!E9)</f>
+        <f>'时间节点计划表'!E9</f>
         <v/>
       </c>
       <c r="E18" s="28">
-        <f>IF('时间节点计划表'!F9="","",'时间节点计划表'!F9)</f>
+        <f>IF(COUNT('时间节点计划表'!F9),'时间节点计划表'!F9,"")</f>
         <v/>
       </c>
       <c r="F18" s="29">
@@ -7566,11 +7513,11 @@
         </is>
       </c>
       <c r="D19" s="23">
-        <f>IF('时间节点计划表'!E10="","",'时间节点计划表'!E10)</f>
+        <f>'时间节点计划表'!E10</f>
         <v/>
       </c>
       <c r="E19" s="23">
-        <f>IF('时间节点计划表'!F10="","",'时间节点计划表'!F10)</f>
+        <f>IF(COUNT('时间节点计划表'!F10),'时间节点计划表'!F10,"")</f>
         <v/>
       </c>
       <c r="F19" s="24" t="inlineStr"/>
@@ -7836,11 +7783,11 @@
         </is>
       </c>
       <c r="D20" s="28">
-        <f>IF('时间节点计划表'!E10="","",'时间节点计划表'!E10)</f>
+        <f>'时间节点计划表'!E10</f>
         <v/>
       </c>
       <c r="E20" s="28">
-        <f>IF('时间节点计划表'!F10="","",'时间节点计划表'!F10)</f>
+        <f>IF(COUNT('时间节点计划表'!F10),'时间节点计划表'!F10,"")</f>
         <v/>
       </c>
       <c r="F20" s="29">
@@ -8109,11 +8056,11 @@
         </is>
       </c>
       <c r="D21" s="23">
-        <f>IF('时间节点计划表'!E11="","",'时间节点计划表'!E11)</f>
+        <f>'时间节点计划表'!E11</f>
         <v/>
       </c>
       <c r="E21" s="23">
-        <f>IF('时间节点计划表'!F11="","",'时间节点计划表'!F11)</f>
+        <f>IF(COUNT('时间节点计划表'!F11),'时间节点计划表'!F11,"")</f>
         <v/>
       </c>
       <c r="F21" s="24" t="inlineStr"/>
@@ -8379,11 +8326,11 @@
         </is>
       </c>
       <c r="D22" s="28">
-        <f>IF('时间节点计划表'!E11="","",'时间节点计划表'!E11)</f>
+        <f>'时间节点计划表'!E11</f>
         <v/>
       </c>
       <c r="E22" s="28">
-        <f>IF('时间节点计划表'!F11="","",'时间节点计划表'!F11)</f>
+        <f>IF(COUNT('时间节点计划表'!F11),'时间节点计划表'!F11,"")</f>
         <v/>
       </c>
       <c r="F22" s="29">
@@ -8652,11 +8599,11 @@
         </is>
       </c>
       <c r="D23" s="23">
-        <f>IF('时间节点计划表'!E12="","",'时间节点计划表'!E12)</f>
+        <f>'时间节点计划表'!E12</f>
         <v/>
       </c>
       <c r="E23" s="23">
-        <f>IF('时间节点计划表'!F12="","",'时间节点计划表'!F12)</f>
+        <f>IF(COUNT('时间节点计划表'!F12),'时间节点计划表'!F12,"")</f>
         <v/>
       </c>
       <c r="F23" s="24" t="inlineStr"/>
@@ -8922,11 +8869,11 @@
         </is>
       </c>
       <c r="D24" s="28">
-        <f>IF('时间节点计划表'!E12="","",'时间节点计划表'!E12)</f>
+        <f>'时间节点计划表'!E12</f>
         <v/>
       </c>
       <c r="E24" s="28">
-        <f>IF('时间节点计划表'!F12="","",'时间节点计划表'!F12)</f>
+        <f>IF(COUNT('时间节点计划表'!F12),'时间节点计划表'!F12,"")</f>
         <v/>
       </c>
       <c r="F24" s="29">
@@ -9195,11 +9142,11 @@
         </is>
       </c>
       <c r="D25" s="23">
-        <f>IF('时间节点计划表'!E13="","",'时间节点计划表'!E13)</f>
+        <f>'时间节点计划表'!E13</f>
         <v/>
       </c>
       <c r="E25" s="23">
-        <f>IF('时间节点计划表'!F13="","",'时间节点计划表'!F13)</f>
+        <f>IF(COUNT('时间节点计划表'!F13),'时间节点计划表'!F13,"")</f>
         <v/>
       </c>
       <c r="F25" s="24" t="inlineStr"/>
@@ -9465,11 +9412,11 @@
         </is>
       </c>
       <c r="D26" s="28">
-        <f>IF('时间节点计划表'!E13="","",'时间节点计划表'!E13)</f>
+        <f>'时间节点计划表'!E13</f>
         <v/>
       </c>
       <c r="E26" s="28">
-        <f>IF('时间节点计划表'!F13="","",'时间节点计划表'!F13)</f>
+        <f>IF(COUNT('时间节点计划表'!F13),'时间节点计划表'!F13,"")</f>
         <v/>
       </c>
       <c r="F26" s="29">
@@ -9738,11 +9685,11 @@
         </is>
       </c>
       <c r="D27" s="23">
-        <f>IF('时间节点计划表'!E14="","",'时间节点计划表'!E14)</f>
+        <f>'时间节点计划表'!E14</f>
         <v/>
       </c>
       <c r="E27" s="23">
-        <f>IF('时间节点计划表'!F14="","",'时间节点计划表'!F14)</f>
+        <f>IF(COUNT('时间节点计划表'!F14),'时间节点计划表'!F14,"")</f>
         <v/>
       </c>
       <c r="F27" s="24" t="inlineStr"/>
@@ -10008,11 +9955,11 @@
         </is>
       </c>
       <c r="D28" s="28">
-        <f>IF('时间节点计划表'!E14="","",'时间节点计划表'!E14)</f>
+        <f>'时间节点计划表'!E14</f>
         <v/>
       </c>
       <c r="E28" s="28">
-        <f>IF('时间节点计划表'!F14="","",'时间节点计划表'!F14)</f>
+        <f>IF(COUNT('时间节点计划表'!F14),'时间节点计划表'!F14,"")</f>
         <v/>
       </c>
       <c r="F28" s="29">
@@ -10281,11 +10228,11 @@
         </is>
       </c>
       <c r="D29" s="23">
-        <f>IF('时间节点计划表'!E15="","",'时间节点计划表'!E15)</f>
+        <f>'时间节点计划表'!E15</f>
         <v/>
       </c>
       <c r="E29" s="23">
-        <f>IF('时间节点计划表'!F15="","",'时间节点计划表'!F15)</f>
+        <f>IF(COUNT('时间节点计划表'!F15),'时间节点计划表'!F15,"")</f>
         <v/>
       </c>
       <c r="F29" s="24" t="inlineStr"/>
@@ -10551,11 +10498,11 @@
         </is>
       </c>
       <c r="D30" s="28">
-        <f>IF('时间节点计划表'!E15="","",'时间节点计划表'!E15)</f>
+        <f>'时间节点计划表'!E15</f>
         <v/>
       </c>
       <c r="E30" s="28">
-        <f>IF('时间节点计划表'!F15="","",'时间节点计划表'!F15)</f>
+        <f>IF(COUNT('时间节点计划表'!F15),'时间节点计划表'!F15,"")</f>
         <v/>
       </c>
       <c r="F30" s="29">
@@ -10824,11 +10771,11 @@
         </is>
       </c>
       <c r="D31" s="23">
-        <f>IF('时间节点计划表'!E16="","",'时间节点计划表'!E16)</f>
+        <f>'时间节点计划表'!E16</f>
         <v/>
       </c>
       <c r="E31" s="23">
-        <f>IF('时间节点计划表'!F16="","",'时间节点计划表'!F16)</f>
+        <f>IF(COUNT('时间节点计划表'!F16),'时间节点计划表'!F16,"")</f>
         <v/>
       </c>
       <c r="F31" s="24" t="inlineStr"/>
@@ -11094,11 +11041,11 @@
         </is>
       </c>
       <c r="D32" s="28">
-        <f>IF('时间节点计划表'!E16="","",'时间节点计划表'!E16)</f>
+        <f>'时间节点计划表'!E16</f>
         <v/>
       </c>
       <c r="E32" s="28">
-        <f>IF('时间节点计划表'!F16="","",'时间节点计划表'!F16)</f>
+        <f>IF(COUNT('时间节点计划表'!F16),'时间节点计划表'!F16,"")</f>
         <v/>
       </c>
       <c r="F32" s="29">
@@ -11367,11 +11314,11 @@
         </is>
       </c>
       <c r="D33" s="23">
-        <f>IF('时间节点计划表'!E17="","",'时间节点计划表'!E17)</f>
+        <f>'时间节点计划表'!E17</f>
         <v/>
       </c>
       <c r="E33" s="23">
-        <f>IF('时间节点计划表'!F17="","",'时间节点计划表'!F17)</f>
+        <f>IF(COUNT('时间节点计划表'!F17),'时间节点计划表'!F17,"")</f>
         <v/>
       </c>
       <c r="F33" s="24" t="inlineStr"/>
@@ -11637,11 +11584,11 @@
         </is>
       </c>
       <c r="D34" s="28">
-        <f>IF('时间节点计划表'!E17="","",'时间节点计划表'!E17)</f>
+        <f>'时间节点计划表'!E17</f>
         <v/>
       </c>
       <c r="E34" s="28">
-        <f>IF('时间节点计划表'!F17="","",'时间节点计划表'!F17)</f>
+        <f>IF(COUNT('时间节点计划表'!F17),'时间节点计划表'!F17,"")</f>
         <v/>
       </c>
       <c r="F34" s="29">
@@ -11910,11 +11857,11 @@
         </is>
       </c>
       <c r="D35" s="23">
-        <f>IF('时间节点计划表'!E18="","",'时间节点计划表'!E18)</f>
+        <f>'时间节点计划表'!E18</f>
         <v/>
       </c>
       <c r="E35" s="23">
-        <f>IF('时间节点计划表'!F18="","",'时间节点计划表'!F18)</f>
+        <f>IF(COUNT('时间节点计划表'!F18),'时间节点计划表'!F18,"")</f>
         <v/>
       </c>
       <c r="F35" s="24" t="inlineStr"/>
@@ -12180,11 +12127,11 @@
         </is>
       </c>
       <c r="D36" s="28">
-        <f>IF('时间节点计划表'!E18="","",'时间节点计划表'!E18)</f>
+        <f>'时间节点计划表'!E18</f>
         <v/>
       </c>
       <c r="E36" s="28">
-        <f>IF('时间节点计划表'!F18="","",'时间节点计划表'!F18)</f>
+        <f>IF(COUNT('时间节点计划表'!F18),'时间节点计划表'!F18,"")</f>
         <v/>
       </c>
       <c r="F36" s="29">
@@ -12453,11 +12400,11 @@
         </is>
       </c>
       <c r="D37" s="23">
-        <f>IF('时间节点计划表'!E19="","",'时间节点计划表'!E19)</f>
+        <f>'时间节点计划表'!E19</f>
         <v/>
       </c>
       <c r="E37" s="23">
-        <f>IF('时间节点计划表'!F19="","",'时间节点计划表'!F19)</f>
+        <f>IF(COUNT('时间节点计划表'!F19),'时间节点计划表'!F19,"")</f>
         <v/>
       </c>
       <c r="F37" s="24" t="inlineStr"/>
@@ -12723,11 +12670,11 @@
         </is>
       </c>
       <c r="D38" s="28">
-        <f>IF('时间节点计划表'!E19="","",'时间节点计划表'!E19)</f>
+        <f>'时间节点计划表'!E19</f>
         <v/>
       </c>
       <c r="E38" s="28">
-        <f>IF('时间节点计划表'!F19="","",'时间节点计划表'!F19)</f>
+        <f>IF(COUNT('时间节点计划表'!F19),'时间节点计划表'!F19,"")</f>
         <v/>
       </c>
       <c r="F38" s="29">
@@ -12996,11 +12943,11 @@
         </is>
       </c>
       <c r="D39" s="23">
-        <f>IF('时间节点计划表'!E20="","",'时间节点计划表'!E20)</f>
+        <f>'时间节点计划表'!E20</f>
         <v/>
       </c>
       <c r="E39" s="23">
-        <f>IF('时间节点计划表'!F20="","",'时间节点计划表'!F20)</f>
+        <f>IF(COUNT('时间节点计划表'!F20),'时间节点计划表'!F20,"")</f>
         <v/>
       </c>
       <c r="F39" s="24" t="inlineStr"/>
@@ -13266,11 +13213,11 @@
         </is>
       </c>
       <c r="D40" s="28">
-        <f>IF('时间节点计划表'!E20="","",'时间节点计划表'!E20)</f>
+        <f>'时间节点计划表'!E20</f>
         <v/>
       </c>
       <c r="E40" s="28">
-        <f>IF('时间节点计划表'!F20="","",'时间节点计划表'!F20)</f>
+        <f>IF(COUNT('时间节点计划表'!F20),'时间节点计划表'!F20,"")</f>
         <v/>
       </c>
       <c r="F40" s="29">
@@ -13539,11 +13486,11 @@
         </is>
       </c>
       <c r="D41" s="23">
-        <f>IF('时间节点计划表'!E21="","",'时间节点计划表'!E21)</f>
+        <f>'时间节点计划表'!E21</f>
         <v/>
       </c>
       <c r="E41" s="23">
-        <f>IF('时间节点计划表'!F21="","",'时间节点计划表'!F21)</f>
+        <f>IF(COUNT('时间节点计划表'!F21),'时间节点计划表'!F21,"")</f>
         <v/>
       </c>
       <c r="F41" s="24" t="inlineStr"/>
@@ -13809,11 +13756,11 @@
         </is>
       </c>
       <c r="D42" s="28">
-        <f>IF('时间节点计划表'!E21="","",'时间节点计划表'!E21)</f>
+        <f>'时间节点计划表'!E21</f>
         <v/>
       </c>
       <c r="E42" s="28">
-        <f>IF('时间节点计划表'!F21="","",'时间节点计划表'!F21)</f>
+        <f>IF(COUNT('时间节点计划表'!F21),'时间节点计划表'!F21,"")</f>
         <v/>
       </c>
       <c r="F42" s="29">
@@ -14082,11 +14029,11 @@
         </is>
       </c>
       <c r="D43" s="23">
-        <f>IF('时间节点计划表'!E22="","",'时间节点计划表'!E22)</f>
+        <f>'时间节点计划表'!E22</f>
         <v/>
       </c>
       <c r="E43" s="23">
-        <f>IF('时间节点计划表'!F22="","",'时间节点计划表'!F22)</f>
+        <f>IF(COUNT('时间节点计划表'!F22),'时间节点计划表'!F22,"")</f>
         <v/>
       </c>
       <c r="F43" s="24" t="inlineStr"/>
@@ -14352,11 +14299,11 @@
         </is>
       </c>
       <c r="D44" s="28">
-        <f>IF('时间节点计划表'!E22="","",'时间节点计划表'!E22)</f>
+        <f>'时间节点计划表'!E22</f>
         <v/>
       </c>
       <c r="E44" s="28">
-        <f>IF('时间节点计划表'!F22="","",'时间节点计划表'!F22)</f>
+        <f>IF(COUNT('时间节点计划表'!F22),'时间节点计划表'!F22,"")</f>
         <v/>
       </c>
       <c r="F44" s="29">
@@ -14625,11 +14572,11 @@
         </is>
       </c>
       <c r="D45" s="23">
-        <f>IF('时间节点计划表'!E23="","",'时间节点计划表'!E23)</f>
+        <f>'时间节点计划表'!E23</f>
         <v/>
       </c>
       <c r="E45" s="23">
-        <f>IF('时间节点计划表'!F23="","",'时间节点计划表'!F23)</f>
+        <f>IF(COUNT('时间节点计划表'!F23),'时间节点计划表'!F23,"")</f>
         <v/>
       </c>
       <c r="F45" s="24" t="inlineStr"/>
@@ -14895,11 +14842,11 @@
         </is>
       </c>
       <c r="D46" s="28">
-        <f>IF('时间节点计划表'!E23="","",'时间节点计划表'!E23)</f>
+        <f>'时间节点计划表'!E23</f>
         <v/>
       </c>
       <c r="E46" s="28">
-        <f>IF('时间节点计划表'!F23="","",'时间节点计划表'!F23)</f>
+        <f>IF(COUNT('时间节点计划表'!F23),'时间节点计划表'!F23,"")</f>
         <v/>
       </c>
       <c r="F46" s="29">
@@ -15168,11 +15115,11 @@
         </is>
       </c>
       <c r="D47" s="23">
-        <f>IF('时间节点计划表'!E24="","",'时间节点计划表'!E24)</f>
+        <f>'时间节点计划表'!E24</f>
         <v/>
       </c>
       <c r="E47" s="23">
-        <f>IF('时间节点计划表'!F24="","",'时间节点计划表'!F24)</f>
+        <f>IF(COUNT('时间节点计划表'!F24),'时间节点计划表'!F24,"")</f>
         <v/>
       </c>
       <c r="F47" s="24" t="inlineStr"/>
@@ -15438,11 +15385,11 @@
         </is>
       </c>
       <c r="D48" s="28">
-        <f>IF('时间节点计划表'!E24="","",'时间节点计划表'!E24)</f>
+        <f>'时间节点计划表'!E24</f>
         <v/>
       </c>
       <c r="E48" s="28">
-        <f>IF('时间节点计划表'!F24="","",'时间节点计划表'!F24)</f>
+        <f>IF(COUNT('时间节点计划表'!F24),'时间节点计划表'!F24,"")</f>
         <v/>
       </c>
       <c r="F48" s="29">
@@ -15711,11 +15658,11 @@
         </is>
       </c>
       <c r="D49" s="23">
-        <f>IF('时间节点计划表'!E25="","",'时间节点计划表'!E25)</f>
+        <f>'时间节点计划表'!E25</f>
         <v/>
       </c>
       <c r="E49" s="23">
-        <f>IF('时间节点计划表'!F25="","",'时间节点计划表'!F25)</f>
+        <f>IF(COUNT('时间节点计划表'!F25),'时间节点计划表'!F25,"")</f>
         <v/>
       </c>
       <c r="F49" s="24" t="inlineStr"/>
@@ -15981,11 +15928,11 @@
         </is>
       </c>
       <c r="D50" s="28">
-        <f>IF('时间节点计划表'!E25="","",'时间节点计划表'!E25)</f>
+        <f>'时间节点计划表'!E25</f>
         <v/>
       </c>
       <c r="E50" s="28">
-        <f>IF('时间节点计划表'!F25="","",'时间节点计划表'!F25)</f>
+        <f>IF(COUNT('时间节点计划表'!F25),'时间节点计划表'!F25,"")</f>
         <v/>
       </c>
       <c r="F50" s="29">
@@ -16254,11 +16201,11 @@
         </is>
       </c>
       <c r="D51" s="23">
-        <f>IF('时间节点计划表'!E26="","",'时间节点计划表'!E26)</f>
+        <f>'时间节点计划表'!E26</f>
         <v/>
       </c>
       <c r="E51" s="23">
-        <f>IF('时间节点计划表'!F26="","",'时间节点计划表'!F26)</f>
+        <f>IF(COUNT('时间节点计划表'!F26),'时间节点计划表'!F26,"")</f>
         <v/>
       </c>
       <c r="F51" s="24" t="inlineStr"/>
@@ -16524,11 +16471,11 @@
         </is>
       </c>
       <c r="D52" s="28">
-        <f>IF('时间节点计划表'!E26="","",'时间节点计划表'!E26)</f>
+        <f>'时间节点计划表'!E26</f>
         <v/>
       </c>
       <c r="E52" s="28">
-        <f>IF('时间节点计划表'!F26="","",'时间节点计划表'!F26)</f>
+        <f>IF(COUNT('时间节点计划表'!F26),'时间节点计划表'!F26,"")</f>
         <v/>
       </c>
       <c r="F52" s="29">
@@ -16797,11 +16744,11 @@
         </is>
       </c>
       <c r="D53" s="23">
-        <f>IF('时间节点计划表'!E27="","",'时间节点计划表'!E27)</f>
+        <f>'时间节点计划表'!E27</f>
         <v/>
       </c>
       <c r="E53" s="23">
-        <f>IF('时间节点计划表'!F27="","",'时间节点计划表'!F27)</f>
+        <f>IF(COUNT('时间节点计划表'!F27),'时间节点计划表'!F27,"")</f>
         <v/>
       </c>
       <c r="F53" s="24" t="inlineStr"/>
@@ -17067,11 +17014,11 @@
         </is>
       </c>
       <c r="D54" s="28">
-        <f>IF('时间节点计划表'!E27="","",'时间节点计划表'!E27)</f>
+        <f>'时间节点计划表'!E27</f>
         <v/>
       </c>
       <c r="E54" s="28">
-        <f>IF('时间节点计划表'!F27="","",'时间节点计划表'!F27)</f>
+        <f>IF(COUNT('时间节点计划表'!F27),'时间节点计划表'!F27,"")</f>
         <v/>
       </c>
       <c r="F54" s="29">
@@ -17340,11 +17287,11 @@
         </is>
       </c>
       <c r="D55" s="23">
-        <f>IF('时间节点计划表'!E28="","",'时间节点计划表'!E28)</f>
+        <f>'时间节点计划表'!E28</f>
         <v/>
       </c>
       <c r="E55" s="23">
-        <f>IF('时间节点计划表'!F28="","",'时间节点计划表'!F28)</f>
+        <f>IF(COUNT('时间节点计划表'!F28),'时间节点计划表'!F28,"")</f>
         <v/>
       </c>
       <c r="F55" s="24" t="inlineStr"/>
@@ -17610,11 +17557,11 @@
         </is>
       </c>
       <c r="D56" s="28">
-        <f>IF('时间节点计划表'!E28="","",'时间节点计划表'!E28)</f>
+        <f>'时间节点计划表'!E28</f>
         <v/>
       </c>
       <c r="E56" s="28">
-        <f>IF('时间节点计划表'!F28="","",'时间节点计划表'!F28)</f>
+        <f>IF(COUNT('时间节点计划表'!F28),'时间节点计划表'!F28,"")</f>
         <v/>
       </c>
       <c r="F56" s="29">
@@ -17883,11 +17830,11 @@
         </is>
       </c>
       <c r="D57" s="23">
-        <f>IF('时间节点计划表'!E29="","",'时间节点计划表'!E29)</f>
+        <f>'时间节点计划表'!E29</f>
         <v/>
       </c>
       <c r="E57" s="23">
-        <f>IF('时间节点计划表'!F29="","",'时间节点计划表'!F29)</f>
+        <f>IF(COUNT('时间节点计划表'!F29),'时间节点计划表'!F29,"")</f>
         <v/>
       </c>
       <c r="F57" s="24" t="inlineStr"/>
@@ -18153,11 +18100,11 @@
         </is>
       </c>
       <c r="D58" s="28">
-        <f>IF('时间节点计划表'!E29="","",'时间节点计划表'!E29)</f>
+        <f>'时间节点计划表'!E29</f>
         <v/>
       </c>
       <c r="E58" s="28">
-        <f>IF('时间节点计划表'!F29="","",'时间节点计划表'!F29)</f>
+        <f>IF(COUNT('时间节点计划表'!F29),'时间节点计划表'!F29,"")</f>
         <v/>
       </c>
       <c r="F58" s="29">
@@ -18426,11 +18373,11 @@
         </is>
       </c>
       <c r="D59" s="23">
-        <f>IF('时间节点计划表'!E30="","",'时间节点计划表'!E30)</f>
+        <f>'时间节点计划表'!E30</f>
         <v/>
       </c>
       <c r="E59" s="23">
-        <f>IF('时间节点计划表'!F30="","",'时间节点计划表'!F30)</f>
+        <f>IF(COUNT('时间节点计划表'!F30),'时间节点计划表'!F30,"")</f>
         <v/>
       </c>
       <c r="F59" s="24" t="inlineStr"/>
@@ -18696,11 +18643,11 @@
         </is>
       </c>
       <c r="D60" s="28">
-        <f>IF('时间节点计划表'!E30="","",'时间节点计划表'!E30)</f>
+        <f>'时间节点计划表'!E30</f>
         <v/>
       </c>
       <c r="E60" s="28">
-        <f>IF('时间节点计划表'!F30="","",'时间节点计划表'!F30)</f>
+        <f>IF(COUNT('时间节点计划表'!F30),'时间节点计划表'!F30,"")</f>
         <v/>
       </c>
       <c r="F60" s="29">
@@ -18969,11 +18916,11 @@
         </is>
       </c>
       <c r="D61" s="23">
-        <f>IF('时间节点计划表'!E31="","",'时间节点计划表'!E31)</f>
+        <f>'时间节点计划表'!E31</f>
         <v/>
       </c>
       <c r="E61" s="23">
-        <f>IF('时间节点计划表'!F31="","",'时间节点计划表'!F31)</f>
+        <f>IF(COUNT('时间节点计划表'!F31),'时间节点计划表'!F31,"")</f>
         <v/>
       </c>
       <c r="F61" s="24" t="inlineStr"/>
@@ -19239,11 +19186,11 @@
         </is>
       </c>
       <c r="D62" s="28">
-        <f>IF('时间节点计划表'!E31="","",'时间节点计划表'!E31)</f>
+        <f>'时间节点计划表'!E31</f>
         <v/>
       </c>
       <c r="E62" s="28">
-        <f>IF('时间节点计划表'!F31="","",'时间节点计划表'!F31)</f>
+        <f>IF(COUNT('时间节点计划表'!F31),'时间节点计划表'!F31,"")</f>
         <v/>
       </c>
       <c r="F62" s="29">
@@ -19512,11 +19459,11 @@
         </is>
       </c>
       <c r="D63" s="23">
-        <f>IF('时间节点计划表'!E32="","",'时间节点计划表'!E32)</f>
+        <f>'时间节点计划表'!E32</f>
         <v/>
       </c>
       <c r="E63" s="23">
-        <f>IF('时间节点计划表'!F32="","",'时间节点计划表'!F32)</f>
+        <f>IF(COUNT('时间节点计划表'!F32),'时间节点计划表'!F32,"")</f>
         <v/>
       </c>
       <c r="F63" s="24" t="inlineStr"/>
@@ -19782,11 +19729,11 @@
         </is>
       </c>
       <c r="D64" s="28">
-        <f>IF('时间节点计划表'!E32="","",'时间节点计划表'!E32)</f>
+        <f>'时间节点计划表'!E32</f>
         <v/>
       </c>
       <c r="E64" s="28">
-        <f>IF('时间节点计划表'!F32="","",'时间节点计划表'!F32)</f>
+        <f>IF(COUNT('时间节点计划表'!F32),'时间节点计划表'!F32,"")</f>
         <v/>
       </c>
       <c r="F64" s="29">
@@ -20055,11 +20002,11 @@
         </is>
       </c>
       <c r="D65" s="23">
-        <f>IF('时间节点计划表'!E33="","",'时间节点计划表'!E33)</f>
+        <f>'时间节点计划表'!E33</f>
         <v/>
       </c>
       <c r="E65" s="23">
-        <f>IF('时间节点计划表'!F33="","",'时间节点计划表'!F33)</f>
+        <f>IF(COUNT('时间节点计划表'!F33),'时间节点计划表'!F33,"")</f>
         <v/>
       </c>
       <c r="F65" s="24" t="inlineStr"/>
@@ -20325,11 +20272,11 @@
         </is>
       </c>
       <c r="D66" s="28">
-        <f>IF('时间节点计划表'!E33="","",'时间节点计划表'!E33)</f>
+        <f>'时间节点计划表'!E33</f>
         <v/>
       </c>
       <c r="E66" s="28">
-        <f>IF('时间节点计划表'!F33="","",'时间节点计划表'!F33)</f>
+        <f>IF(COUNT('时间节点计划表'!F33),'时间节点计划表'!F33,"")</f>
         <v/>
       </c>
       <c r="F66" s="29">
@@ -20598,11 +20545,11 @@
         </is>
       </c>
       <c r="D67" s="23">
-        <f>IF('时间节点计划表'!E34="","",'时间节点计划表'!E34)</f>
+        <f>'时间节点计划表'!E34</f>
         <v/>
       </c>
       <c r="E67" s="23">
-        <f>IF('时间节点计划表'!F34="","",'时间节点计划表'!F34)</f>
+        <f>IF(COUNT('时间节点计划表'!F34),'时间节点计划表'!F34,"")</f>
         <v/>
       </c>
       <c r="F67" s="24" t="inlineStr"/>
@@ -20868,11 +20815,11 @@
         </is>
       </c>
       <c r="D68" s="28">
-        <f>IF('时间节点计划表'!E34="","",'时间节点计划表'!E34)</f>
+        <f>'时间节点计划表'!E34</f>
         <v/>
       </c>
       <c r="E68" s="28">
-        <f>IF('时间节点计划表'!F34="","",'时间节点计划表'!F34)</f>
+        <f>IF(COUNT('时间节点计划表'!F34),'时间节点计划表'!F34,"")</f>
         <v/>
       </c>
       <c r="F68" s="29">
@@ -21141,11 +21088,11 @@
         </is>
       </c>
       <c r="D69" s="23">
-        <f>IF('时间节点计划表'!E35="","",'时间节点计划表'!E35)</f>
+        <f>'时间节点计划表'!E35</f>
         <v/>
       </c>
       <c r="E69" s="23">
-        <f>IF('时间节点计划表'!F35="","",'时间节点计划表'!F35)</f>
+        <f>IF(COUNT('时间节点计划表'!F35),'时间节点计划表'!F35,"")</f>
         <v/>
       </c>
       <c r="F69" s="24" t="inlineStr"/>
@@ -21411,11 +21358,11 @@
         </is>
       </c>
       <c r="D70" s="28">
-        <f>IF('时间节点计划表'!E35="","",'时间节点计划表'!E35)</f>
+        <f>'时间节点计划表'!E35</f>
         <v/>
       </c>
       <c r="E70" s="28">
-        <f>IF('时间节点计划表'!F35="","",'时间节点计划表'!F35)</f>
+        <f>IF(COUNT('时间节点计划表'!F35),'时间节点计划表'!F35,"")</f>
         <v/>
       </c>
       <c r="F70" s="29">
@@ -21684,11 +21631,11 @@
         </is>
       </c>
       <c r="D71" s="23">
-        <f>IF('时间节点计划表'!E36="","",'时间节点计划表'!E36)</f>
+        <f>'时间节点计划表'!E36</f>
         <v/>
       </c>
       <c r="E71" s="23">
-        <f>IF('时间节点计划表'!F36="","",'时间节点计划表'!F36)</f>
+        <f>IF(COUNT('时间节点计划表'!F36),'时间节点计划表'!F36,"")</f>
         <v/>
       </c>
       <c r="F71" s="24" t="inlineStr"/>
@@ -21954,11 +21901,11 @@
         </is>
       </c>
       <c r="D72" s="28">
-        <f>IF('时间节点计划表'!E36="","",'时间节点计划表'!E36)</f>
+        <f>'时间节点计划表'!E36</f>
         <v/>
       </c>
       <c r="E72" s="28">
-        <f>IF('时间节点计划表'!F36="","",'时间节点计划表'!F36)</f>
+        <f>IF(COUNT('时间节点计划表'!F36),'时间节点计划表'!F36,"")</f>
         <v/>
       </c>
       <c r="F72" s="29">
@@ -22227,11 +22174,11 @@
         </is>
       </c>
       <c r="D73" s="23">
-        <f>IF('时间节点计划表'!E37="","",'时间节点计划表'!E37)</f>
+        <f>'时间节点计划表'!E37</f>
         <v/>
       </c>
       <c r="E73" s="23">
-        <f>IF('时间节点计划表'!F37="","",'时间节点计划表'!F37)</f>
+        <f>IF(COUNT('时间节点计划表'!F37),'时间节点计划表'!F37,"")</f>
         <v/>
       </c>
       <c r="F73" s="24" t="inlineStr"/>
@@ -22497,11 +22444,11 @@
         </is>
       </c>
       <c r="D74" s="28">
-        <f>IF('时间节点计划表'!E37="","",'时间节点计划表'!E37)</f>
+        <f>'时间节点计划表'!E37</f>
         <v/>
       </c>
       <c r="E74" s="28">
-        <f>IF('时间节点计划表'!F37="","",'时间节点计划表'!F37)</f>
+        <f>IF(COUNT('时间节点计划表'!F37),'时间节点计划表'!F37,"")</f>
         <v/>
       </c>
       <c r="F74" s="29">
@@ -22770,11 +22717,11 @@
         </is>
       </c>
       <c r="D75" s="23">
-        <f>IF('时间节点计划表'!E38="","",'时间节点计划表'!E38)</f>
+        <f>'时间节点计划表'!E38</f>
         <v/>
       </c>
       <c r="E75" s="23">
-        <f>IF('时间节点计划表'!F38="","",'时间节点计划表'!F38)</f>
+        <f>IF(COUNT('时间节点计划表'!F38),'时间节点计划表'!F38,"")</f>
         <v/>
       </c>
       <c r="F75" s="24" t="inlineStr"/>
@@ -23040,11 +22987,11 @@
         </is>
       </c>
       <c r="D76" s="28">
-        <f>IF('时间节点计划表'!E38="","",'时间节点计划表'!E38)</f>
+        <f>'时间节点计划表'!E38</f>
         <v/>
       </c>
       <c r="E76" s="28">
-        <f>IF('时间节点计划表'!F38="","",'时间节点计划表'!F38)</f>
+        <f>IF(COUNT('时间节点计划表'!F38),'时间节点计划表'!F38,"")</f>
         <v/>
       </c>
       <c r="F76" s="29">
@@ -23313,11 +23260,11 @@
         </is>
       </c>
       <c r="D77" s="23">
-        <f>IF('时间节点计划表'!E39="","",'时间节点计划表'!E39)</f>
+        <f>'时间节点计划表'!E39</f>
         <v/>
       </c>
       <c r="E77" s="23">
-        <f>IF('时间节点计划表'!F39="","",'时间节点计划表'!F39)</f>
+        <f>IF(COUNT('时间节点计划表'!F39),'时间节点计划表'!F39,"")</f>
         <v/>
       </c>
       <c r="F77" s="24" t="inlineStr"/>
@@ -23583,11 +23530,11 @@
         </is>
       </c>
       <c r="D78" s="28">
-        <f>IF('时间节点计划表'!E39="","",'时间节点计划表'!E39)</f>
+        <f>'时间节点计划表'!E39</f>
         <v/>
       </c>
       <c r="E78" s="28">
-        <f>IF('时间节点计划表'!F39="","",'时间节点计划表'!F39)</f>
+        <f>IF(COUNT('时间节点计划表'!F39),'时间节点计划表'!F39,"")</f>
         <v/>
       </c>
       <c r="F78" s="29">
@@ -23856,11 +23803,11 @@
         </is>
       </c>
       <c r="D79" s="23">
-        <f>IF('时间节点计划表'!E40="","",'时间节点计划表'!E40)</f>
+        <f>'时间节点计划表'!E40</f>
         <v/>
       </c>
       <c r="E79" s="23">
-        <f>IF('时间节点计划表'!F40="","",'时间节点计划表'!F40)</f>
+        <f>IF(COUNT('时间节点计划表'!F40),'时间节点计划表'!F40,"")</f>
         <v/>
       </c>
       <c r="F79" s="24" t="inlineStr"/>
@@ -24126,11 +24073,11 @@
         </is>
       </c>
       <c r="D80" s="28">
-        <f>IF('时间节点计划表'!E40="","",'时间节点计划表'!E40)</f>
+        <f>'时间节点计划表'!E40</f>
         <v/>
       </c>
       <c r="E80" s="28">
-        <f>IF('时间节点计划表'!F40="","",'时间节点计划表'!F40)</f>
+        <f>IF(COUNT('时间节点计划表'!F40),'时间节点计划表'!F40,"")</f>
         <v/>
       </c>
       <c r="F80" s="29">
@@ -24399,11 +24346,11 @@
         </is>
       </c>
       <c r="D81" s="23">
-        <f>IF('时间节点计划表'!E41="","",'时间节点计划表'!E41)</f>
+        <f>'时间节点计划表'!E41</f>
         <v/>
       </c>
       <c r="E81" s="23">
-        <f>IF('时间节点计划表'!F41="","",'时间节点计划表'!F41)</f>
+        <f>IF(COUNT('时间节点计划表'!F41),'时间节点计划表'!F41,"")</f>
         <v/>
       </c>
       <c r="F81" s="24" t="inlineStr"/>
@@ -24669,11 +24616,11 @@
         </is>
       </c>
       <c r="D82" s="28">
-        <f>IF('时间节点计划表'!E41="","",'时间节点计划表'!E41)</f>
+        <f>'时间节点计划表'!E41</f>
         <v/>
       </c>
       <c r="E82" s="28">
-        <f>IF('时间节点计划表'!F41="","",'时间节点计划表'!F41)</f>
+        <f>IF(COUNT('时间节点计划表'!F41),'时间节点计划表'!F41,"")</f>
         <v/>
       </c>
       <c r="F82" s="29">
@@ -24942,11 +24889,11 @@
         </is>
       </c>
       <c r="D83" s="23">
-        <f>IF('时间节点计划表'!E42="","",'时间节点计划表'!E42)</f>
+        <f>'时间节点计划表'!E42</f>
         <v/>
       </c>
       <c r="E83" s="23">
-        <f>IF('时间节点计划表'!F42="","",'时间节点计划表'!F42)</f>
+        <f>IF(COUNT('时间节点计划表'!F42),'时间节点计划表'!F42,"")</f>
         <v/>
       </c>
       <c r="F83" s="24" t="inlineStr"/>
@@ -25212,11 +25159,11 @@
         </is>
       </c>
       <c r="D84" s="28">
-        <f>IF('时间节点计划表'!E42="","",'时间节点计划表'!E42)</f>
+        <f>'时间节点计划表'!E42</f>
         <v/>
       </c>
       <c r="E84" s="28">
-        <f>IF('时间节点计划表'!F42="","",'时间节点计划表'!F42)</f>
+        <f>IF(COUNT('时间节点计划表'!F42),'时间节点计划表'!F42,"")</f>
         <v/>
       </c>
       <c r="F84" s="29">
@@ -25485,11 +25432,11 @@
         </is>
       </c>
       <c r="D85" s="23">
-        <f>IF('时间节点计划表'!E43="","",'时间节点计划表'!E43)</f>
+        <f>'时间节点计划表'!E43</f>
         <v/>
       </c>
       <c r="E85" s="23">
-        <f>IF('时间节点计划表'!F43="","",'时间节点计划表'!F43)</f>
+        <f>IF(COUNT('时间节点计划表'!F43),'时间节点计划表'!F43,"")</f>
         <v/>
       </c>
       <c r="F85" s="24" t="inlineStr"/>
@@ -25755,11 +25702,11 @@
         </is>
       </c>
       <c r="D86" s="28">
-        <f>IF('时间节点计划表'!E43="","",'时间节点计划表'!E43)</f>
+        <f>'时间节点计划表'!E43</f>
         <v/>
       </c>
       <c r="E86" s="28">
-        <f>IF('时间节点计划表'!F43="","",'时间节点计划表'!F43)</f>
+        <f>IF(COUNT('时间节点计划表'!F43),'时间节点计划表'!F43,"")</f>
         <v/>
       </c>
       <c r="F86" s="29">
@@ -26028,11 +25975,11 @@
         </is>
       </c>
       <c r="D87" s="23">
-        <f>IF('时间节点计划表'!E44="","",'时间节点计划表'!E44)</f>
+        <f>'时间节点计划表'!E44</f>
         <v/>
       </c>
       <c r="E87" s="23">
-        <f>IF('时间节点计划表'!F44="","",'时间节点计划表'!F44)</f>
+        <f>IF(COUNT('时间节点计划表'!F44),'时间节点计划表'!F44,"")</f>
         <v/>
       </c>
       <c r="F87" s="24" t="inlineStr"/>
@@ -26298,11 +26245,11 @@
         </is>
       </c>
       <c r="D88" s="28">
-        <f>IF('时间节点计划表'!E44="","",'时间节点计划表'!E44)</f>
+        <f>'时间节点计划表'!E44</f>
         <v/>
       </c>
       <c r="E88" s="28">
-        <f>IF('时间节点计划表'!F44="","",'时间节点计划表'!F44)</f>
+        <f>IF(COUNT('时间节点计划表'!F44),'时间节点计划表'!F44,"")</f>
         <v/>
       </c>
       <c r="F88" s="29">
@@ -26571,11 +26518,11 @@
         </is>
       </c>
       <c r="D89" s="23">
-        <f>IF('时间节点计划表'!E45="","",'时间节点计划表'!E45)</f>
+        <f>'时间节点计划表'!E45</f>
         <v/>
       </c>
       <c r="E89" s="23">
-        <f>IF('时间节点计划表'!F45="","",'时间节点计划表'!F45)</f>
+        <f>IF(COUNT('时间节点计划表'!F45),'时间节点计划表'!F45,"")</f>
         <v/>
       </c>
       <c r="F89" s="24" t="inlineStr"/>
@@ -26841,11 +26788,11 @@
         </is>
       </c>
       <c r="D90" s="28">
-        <f>IF('时间节点计划表'!E45="","",'时间节点计划表'!E45)</f>
+        <f>'时间节点计划表'!E45</f>
         <v/>
       </c>
       <c r="E90" s="28">
-        <f>IF('时间节点计划表'!F45="","",'时间节点计划表'!F45)</f>
+        <f>IF(COUNT('时间节点计划表'!F45),'时间节点计划表'!F45,"")</f>
         <v/>
       </c>
       <c r="F90" s="29">
@@ -27146,44 +27093,6 @@
       <formula>AND($A3="实际",ISNUMBER(G3),$E3&lt;$D3)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A90">
-    <cfRule type="expression" priority="5" dxfId="7">
-      <formula>AND($A3="预估",ISNUMBER($D3))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="8">
-      <formula>AND($A3="实际",ISNUMBER($E3),$E3&gt;$D3)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="9">
-      <formula>AND($A3="实际",ISNUMBER($E3),$E3&lt;$D3)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="10">
-      <formula>AND($A3="实际",ISNUMBER($E3),$E3=$D3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D90">
-    <cfRule type="expression" priority="9" dxfId="7">
-      <formula>ISNUMBER(D3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E90">
-    <cfRule type="expression" priority="10" dxfId="8">
-      <formula>AND(ISNUMBER(E3),E3&gt;D3)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="9">
-      <formula>AND(ISNUMBER(E3),E3&lt;D3)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="10">
-      <formula>AND(ISNUMBER(E3),E3=D3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F90">
-    <cfRule type="expression" priority="13" dxfId="8">
-      <formula>AND(ISNUMBER(F3),F3&gt;0)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="9">
-      <formula>AND(ISNUMBER(F3),F3&lt;0)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8"/>
 </worksheet>

</xml_diff>